<commit_message>
revision del 2026-08-18: ortografia y conteo de borradores
</commit_message>
<xml_diff>
--- a/2026-08-18/barrido-2026-08-18.xlsx
+++ b/2026-08-18/barrido-2026-08-18.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Alvaro Ml. Garcia Segura (HeyReach 214686) + LinkedIn + es_es</t>
+          <t>Álvaro Ml. García Segura (HeyReach 214686) + LinkedIn + es_es</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -773,13 +773,13 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>peticion del contacto, en pregunta directa</t>
+          <t>petición del contacto, en pregunta directa</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
           <t>acuse corto con su nombre y petición del contacto de la referida. Sin material, sin casos y sin propuesta de reunión, según referidos.md 1 bis y la fila Wrong Person de la matriz
-— apertura: acuse corto (Entendido + nombre) | 1ª frase: 2 palabras | qué hacemos: no entra: la rama Wrong Person solo pide el contacto y el material está prohibido aquí | cierre: petición del contacto formulada como pregunta directa | frases: 2</t>
+· apertura: acuse corto (Entendido + nombre) | 1ª frase: 2 palabras | qué hacemos: no entra: la rama Wrong Person solo pide el contacto y el material está prohibido aquí | cierre: petición del contacto formulada como pregunta directa | frases: 2</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -831,7 +831,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Alvaro Ml. Garcia Segura (HeyReach 214686) + LinkedIn + es_es</t>
+          <t>Álvaro Ml. García Segura (HeyReach 214686) + LinkedIn + es_es</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>ANGULO: sin senal publica
+          <t>ANGULO: sin señal publica
 FUENTE: la empresa cargada en la campaña es Zappas y el headline del lead dice Mascotas Ávila, y ninguna búsqueda resuelve cuál es la del hilo. Lo encontrado, 24 tiendas de Mascotas Ávila en Cádiz, Sevilla y Málaga con cinco aperturas en 2025 (elconciso.es), no se puede atribuir con seguridad, así que no entra en el mensaje. El material sale del propio hilo
 FECHA DE LA SENAL: 
 ENCAJE: adyacente
@@ -933,7 +933,7 @@
       <c r="X3" s="3" t="inlineStr">
         <is>
           <t>descargo de intención, qué hacemos en frase aparte (no colgado de dos puntos) y binaria de semilla. No se nombra ni se ataca al proveedor y no se repite la palabra que usó el lead, vetada por marca
-— apertura: nombre + descargo de intención | 1ª frase: 7 palabras | qué hacemos: frase propia que arranca con el sujeto SERDEL, justo después del descargo | cierre: pregunta binaria de semilla apuntando a la próxima decisión | frases: 4</t>
+· apertura: nombre + descargo de intención | 1ª frase: 7 palabras | qué hacemos: frase propia que arranca con el sujeto SERDEL, justo después del descargo | cierre: pregunta binaria de semilla apuntando a la próxima decisión | frases: 4</t>
         </is>
       </c>
       <c r="Y3" s="3" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Alvaro Ml. Garcia Segura (HeyReach 214686) + LinkedIn + es_es</t>
+          <t>Álvaro Ml. García Segura (HeyReach 214686) + LinkedIn + es_es</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>ANGULO: sin senal publica
+          <t>ANGULO: sin señal publica
 FUENTE: Otrura es una marca española de moda de autor que produce bajo demanda, fundada por Sergio de Lázaro y Verónica Abián, con venta al consumidor final y salto al multimarca (modaes.com, 2021-10). No hay señal dentro de los últimos doce meses y otrura.com no se dejó leer (robots). El material del mensaje sale del propio hilo: edificio BIC y patrimonio
 FECHA DE LA SENAL: 
 ENCAJE: pleno
@@ -1086,7 +1086,7 @@
       <c r="X4" s="2" t="inlineStr">
         <is>
           <t>movimiento de tres tiempos: acuse anclado al dato del hilo marcado como suposición, porqué de la pregunta con el qué hacemos en frase aparte, y binaria. No se afirma experiencia en BIC ni en patrimonio porque no está en la ficha
-— apertura: referencia al dato del hilo (patrimonio), en condicional | 1ª frase: 17 palabras | qué hacemos: dentro del porqué de la pregunta anterior, en frase propia y sin dos puntos | cierre: pregunta binaria de intención apuntando al siguiente local | frases: 4</t>
+· apertura: referencia al dato del hilo (patrimonio), en condicional | 1ª frase: 17 palabras | qué hacemos: dentro del porqué de la pregunta anterior, en frase propia y sin dos puntos | cierre: pregunta binaria de intención apuntando al siguiente local | frases: 4</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Jose Luis Díaz Mariscal</t>
+          <t>José Luis Díaz Mariscal</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Alvaro Ml. Garcia Segura (HeyReach 214686) + LinkedIn + es_es</t>
+          <t>Álvaro Ml. García Segura (HeyReach 214686) + LinkedIn + es_es</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>Jose Luis, me quedo con tu correo y te escribo por ahí. Que cada socio responda de su plaza no lo veo un problema. SERDEL puede funcionar como el departamento de arquitectura externo del grupo, con un mismo interlocutor para proyecto, licencias y dirección de obra.</t>
+          <t>José Luis, me quedo con tu correo y te escribo por ahí. Que cada socio responda de su plaza no lo veo un problema. SERDEL puede funcionar como el departamento de arquitectura externo del grupo, con un mismo interlocutor para proyecto, licencias y dirección de obra.</t>
         </is>
       </c>
       <c r="U5" s="3" t="inlineStr">
@@ -1243,7 +1243,7 @@
       <c r="X5" s="3" t="inlineStr">
         <is>
           <t>primero lo que pidió (el cambio de canal), después posicionamiento sin detalle y parada. Sin alcance, sin plazos, sin tarifas, sin duración de reunión y sin prometer qué hará ni cuándo otra persona
-— apertura: nombre + compromiso de canal | 1ª frase: 12 palabras | qué hacemos: tercera frase, arrancando con el sujeto SERDEL, como posicionamiento y no como alcance | cierre: afirmación de posicionamiento, sin pregunta y sin CTA propio | frases: 3</t>
+· apertura: nombre + compromiso de canal | 1ª frase: 12 palabras | qué hacemos: tercera frase, arrancando con el sujeto SERDEL, como posicionamiento y no como alcance | cierre: afirmación de posicionamiento, sin pregunta y sin CTA propio | frases: 3</t>
         </is>
       </c>
       <c r="Y5" s="3" t="inlineStr">
@@ -1399,7 +1399,7 @@
       <c r="X6" s="2" t="inlineStr">
         <is>
           <t>n/a
-— apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
+· apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1451,7 +1451,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Alvaro Pujales Lopez, HeyReach sender_id 214090, LinkedIn, es_es (perfil operado por Carlos)</t>
+          <t>Álvaro Pujales Lopez, HeyReach sender_id 214090, LinkedIn, es_es (perfil operado por Carlos)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Merece continuidad. Dice que no es la persona adecuada pero deja la empresa viva y senala el departamento correcto (circuitos culturales), asi que hay accion concreta: pedir el contacto. No es cierre porque la empresa encaja de pleno, y no es acuse porque deja algo abierto.</t>
+          <t>Merece continuidad. Dice que no es la persona adecuada pero deja la empresa viva y senala el departamento correcto (circuitos culturales), así que hay accion concreta: pedir el contacto. No es cierre porque la empresa encaja de pleno, y no es acuse porque deja algo abierto.</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -1553,18 +1553,18 @@
       <c r="X7" s="3" t="inlineStr">
         <is>
           <t>pregunta directa antepuesta, porqué con la ventaja del contrato, ofrecimiento de hacer el puente
-— apertura: pregunta directa + vocativo | 1ª frase: 6 palabras | qué hacemos: dentro del porqué (Te lo pregunto porque...) | cierre: afirmación con oferta, sin pregunta | frases: 3
-— REESCRITO EN CONTROL DE LOTE: sí: la apertura original era acuse corto con vocativo (Entendido, Gloria), la misma forma que S1 y C1</t>
+· apertura: pregunta directa + vocativo | 1ª frase: 6 palabras | qué hacemos: dentro del porqué (Te lo pregunto porque...) | cierre: afirmación con oferta, sin pregunta | frases: 3
+· REESCRITO EN CONTROL DE LOTE: sí: la apertura original era acuse corto con vocativo (Entendido, Gloria), la misma forma que S1 y C1</t>
         </is>
       </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>Alvaro Pujales Lopez, es_es, tuteo a la persona y vosotros a la empresa, tono que se disculpa por interrumpir. Sin signos de apertura, sin guion largo. LinkedIn no lleva firma.</t>
+          <t>Álvaro Pujales Lopez, es_es, tuteo a la persona y vosotros a la empresa, tono que se disculpa por interrumpir. Sin signos de apertura, sin guion largo. LinkedIn no lleva firma.</t>
         </is>
       </c>
       <c r="Z7" s="3" t="inlineStr">
         <is>
-          <t>Si no da el contacto, toque 1 a 3 dias laborables (2026-08-21) segun followup_ventana_dias=3, tope 4 toques. Si sigue sin darlo tras el segundo toque, Lukewarm.</t>
+          <t>Si no da el contacto, toque 1 a 3 dias laborables (2026-08-21) según followup_ventana_dias=3, tope 4 toques. Si sigue sin darlo tras el segundo toque, Lukewarm.</t>
         </is>
       </c>
       <c r="AA7" s="3" t="inlineStr">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="AB7" s="3" t="inlineStr">
         <is>
-          <t>Media, asi que circuito de aprobacion en Slack de avisos.md. Con aprobacion_manual=true de Offitravel pasaria por aprobacion igual aunque fuese alta. En esta pasada en seco no sale nada: sin envio, sin tag, sin traza.</t>
+          <t>Media, así que circuito de aprobacion en Slack de avisos.md. Con aprobacion_manual=true de Offitravel pasaria por aprobacion igual aunque fuese alta. En esta pasada en seco no sale nada: sin envio, sin tag, sin traza.</t>
         </is>
       </c>
       <c r="AC7" s="3" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Jose Arozarena</t>
+          <t>José Arozarena</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Alvaro Pujales Lopez, HeyReach sender_id 214090, LinkedIn, es_es (perfil operado por Carlos)</t>
+          <t>Álvaro Pujales Lopez, HeyReach sender_id 214090, LinkedIn, es_es (perfil operado por Carlos)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Merece continuidad y es el mejor hilo de los cuatro. Contesta la pregunta del M1 (van por carretera) y ademas declara intencion sin que se la pidamos (nos gustaria hacer parte en tren). Son dos mensajes seguidos suyos, el ultimo es el que manda.</t>
+          <t>Merece continuidad y es el mejor hilo de los cuatro. Contesta la pregunta del M1 (van por carretera) y además declara intencion sin que se la pidamos (nos gustaria hacer parte en tren). Son dos mensajes seguidos suyos, el ultimo es el que manda.</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1671,8 +1671,8 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>ANGULO: sin senal publica
-FUENTE: web de la empresa (amigotours.com) y ficha de El Economista de enero de 2024, fuera de la ventana de doce meses. Lo que si queda verificado por la web: operan mas de 400 tours propios en Espana con guias locales y venden a viajero final, no a agencias
+          <t>ANGULO: sin señal publica
+FUENTE: web de la empresa (amigotours.com) y ficha de El Economista de enero de 2024, fuera de la ventana de doce meses. Lo que si queda verificado por la web: operan más de 400 tours propios en España con guias locales y venden a viajero final, no a agencias
 FECHA DE LA SENAL: sin fecha dentro de la ventana de 12 meses
 ENCAJE: pleno
 ROL: decide
@@ -1687,7 +1687,7 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>Que queráis meter tren es justo por donde entramos, Jose. Te preguntaba porque el precio del billete es lo que más nota el viajero, y ahí pesa el contrato que tengas con Renfe. Si os sirve que le pongamos el tren a lo que ya vendéis, lo vemos en una ruta de las que ya movéis?</t>
+          <t>Que queráis meter tren es justo por donde entramos, José. Te preguntaba porque el precio del billete es lo que más nota el viajero, y ahí pesa el contrato que tengas con Renfe. Si os sirve que le pongamos el tren a lo que ya vendéis, lo vemos en una ruta de las que ya movéis?</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
@@ -1707,13 +1707,13 @@
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>Apertura por el dato que el propio lead puso encima de la mesa, porque el peldano 3 no genera mensaje propio y el coste se nombra dentro del porque (fila de la ficha: el tren es donde esta la diferencia de precio que el viajero nota). El que hacemos entra como subordinada condicional para no repetir la forma de O1. Cierra con binaria de intencion, no con reunion: modo handoff y el CTA comercial es de Alvaro Pujales. Como vende a viajero final y no a agencias, la frase se dice en terminos de lo que el ya vende al viajero, no de reventa de catalogo (enriquecimiento.md 0 ter).
-— apertura: entrada por el dato del lead | 1ª frase: 10 palabras | qué hacemos: subordinada condicional (Si os sirve que...) | cierre: binaria de si o no | frases: 3</t>
+          <t>Apertura por el dato que el propio lead puso encima de la mesa, porque el peldano 3 no genera mensaje propio y el coste se nombra dentro del porque (fila de la ficha: el tren es donde esta la diferencia de precio que el viajero nota). El que hacemos entra como subordinada condicional para no repetir la forma de O1. Cierra con binaria de intencion, no con reunion: modo handoff y el CTA comercial es de Álvaro Pujales. Como vende a viajero final y no a agencias, la frase se dice en terminos de lo que el ya vende al viajero, no de reventa de catalogo (enriquecimiento.md 0 ter).
+· apertura: entrada por el dato del lead | 1ª frase: 10 palabras | qué hacemos: subordinada condicional (Si os sirve que...) | cierre: binaria de si o no | frases: 3</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>Alvaro Pujales Lopez, es_es, tuteo y vosotros. Sin signos de apertura, sin guion largo, sin prueba social porque activos.md prohibe citar agencias.</t>
+          <t>Álvaro Pujales Lopez, es_es, tuteo y vosotros. Sin signos de apertura, sin guion largo, sin prueba social porque activos.md prohíbe citar agencias.</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
-          <t>Media, asi que circuito de aprobacion en Slack. Con aprobacion_manual=true pasaria por aprobacion igual. En esta pasada en seco no sale nada.</t>
+          <t>Media, así que circuito de aprobacion en Slack. Con aprobacion_manual=true pasaria por aprobacion igual. En esta pasada en seco no sale nada.</t>
         </is>
       </c>
       <c r="AC8" s="2" t="inlineStr">
@@ -1810,7 +1810,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Acuse puro. Nuestro toque anterior ya era un cierre cordial (aqui estamos cuando surja) y el lead responde agradeciendo, sin pedir nada, sin pregunta y sin dejar nada abierto. No es punto del arbol: no se redacta. No es D porque 47 dias no llegan al umbral de 90 de hilo dormido.</t>
+          <t>Acuse puro. Nuestro toque anterior ya era un cierre cordial (aquí estamos cuando surja) y el lead responde agradeciendo, sin pedir nada, sin pregunta y sin dejar nada abierto. No es punto del arbol: no se redacta. No es D porque 47 dias no llegan al umbral de 90 de hilo dormido.</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>Espera. El tag lo fija el mensaje con sustancia del 29 de junio (foco en Oman, no expanden portfolio de Espana, nos tendran en cuenta si sale un proyecto ferroviario). Hay trigger de evento aunque no hay fecha, asi que Bad Timing gana a Lukewarm por la regla 8. El acuse del 2 de julio no cambia el tag ni el stage (regla de prioridad 5, no se retrocede en el funnel).</t>
+          <t>Espera. El tag lo fija el mensaje con sustancia del 29 de junio (foco en Oman, no expanden portfolio de España, nos tendran en cuenta sí sale un proyecto ferroviario). Hay trigger de evento aunque no hay fecha, así que Bad Timing gana a Lukewarm por la regla 8. El acuse del 2 de julio no cambia el tag ni el stage (regla de prioridad 5, no se retrocede en el funnel).</t>
         </is>
       </c>
       <c r="P9" s="3" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>ANGULO: no aplica, grupo C: enriquecimiento.md seccion 2 excluye de investigacion lo que no es punto del arbol
+          <t>ANGULO: no aplica, grupo C: enriquecimiento.md sección 2 excluye de investigacion lo que no es punto del arbol
 FUENTE: solo lo que trae la firma del propio correo: Co-Founder, Small-Group Specialist, B2B White-Label Partner, Madrid, y entrega operativa a traves de un DMC local licenciado
 FECHA DE LA SENAL: no aplica
 ENCAJE: adyacente
@@ -1867,8 +1867,8 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>Sin mensaje. Acuse puro que cierra el hilo. Lo unico que toca es el tag y la traza, y en pasada en seco tampoco eso.
-— apertura: no aplica, sin borrador | 1ª frase: 0 palabras | qué hacemos: no aplica | cierre: no aplica | frases: 0</t>
+          <t>Sin mensaje. Acuse puro que cierra el hilo. Lo único que toca es el tag y la traza, y en pasada en seco tampoco eso.
+· apertura: no aplica, sin borrador | 1ª frase: 0 palabras | qué hacemos: no aplica | cierre: no aplica | frases: 0</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="Z9" s="3" t="inlineStr">
         <is>
-          <t>Ninguna. Bad Timing sin fecha concreta, se reactiva por trigger (proyecto o requerimiento ferroviario en Espana), y followup.md prohibe insistir antes. Ademas el hilo queda fuera por moreno_activo_desde.</t>
+          <t>Ninguna. Bad Timing sin fecha concreta, se reactiva por trigger (proyecto o requerimiento ferroviario en España), y followup.md prohíbe insistir antes. Además el hilo queda fuera por moreno_activo_desde.</t>
         </is>
       </c>
       <c r="AA9" s="3" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="AB9" s="3" t="inlineStr">
         <is>
-          <t>Ninguna accion. Grupo C: no se responde. En un barrido real solo se aplicaria tag y traza, y aqui ni eso.</t>
+          <t>Ninguna accion. Grupo C: no se responde. En un barrido real solo se aplicaria tag y traza, y aquí ni eso.</t>
         </is>
       </c>
       <c r="AC9" s="3" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Parece cierre y la ficha dice que no lo es. icp.md declara literalmente que nosotros no manejamos tren es una apertura y no un descarte, y tags.md recoge ese sub caso con el nombre de Offitravel dentro. Ademas la investigacion desmiente la premisa: su web no vende solo habitacion suelta, vende escapadas. Merece un turno mas, y ese turno no es nuestro sino de Alvaro Pujales.</t>
+          <t>Parece cierre y la ficha dice que no lo es. icp.md declara literalmente que nosotros no manejamos tren es una apertura y no un descarte, y tags.md recoge ese sub caso con el nombre de Offitravel dentro. Además la investigacion desmiente la premisa: su web no vende solo habitación suelta, vende escapadas. Merece un turno mas, y ese turno no es nuestro sino de Álvaro Pujales.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1980,7 +1980,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Conversacion. Has Provider manda diferenciador en positivo sin atacar y cierre segun el modo del cliente. En handoff con politica_dudas=deriva y con la prohibicion de generar cuerpo de correo, ese cierre es la derivacion.</t>
+          <t>Conversacion. Has Provider manda diferenciador en positivo sin atacar y cierre según el modo del cliente. En handoff con politica_dudas=deriva y con la prohibicion de generar cuerpo de correo, ese cierre es la derivación.</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>ANGULO: su propia web comercializa escapadas ademas de habitacion suelta, o sea que ya empaquetan, que es justo el encaje que icp.md declara pleno (quien empaqueta hoteles y quiere armar paquetes)
+          <t>ANGULO: su propia web comercializa escapadas además de habitación suelta, o sea que ya empaquetan, que es justo el encaje que icp.md declara pleno (quien empaqueta hoteles y quiere armar paquetes)
 FUENTE: web de la empresa (granshotelsdecatalunya.com)
 FECHA DE LA SENAL: sin fecha, contenido vivo de la web
 ENCAJE: pleno
@@ -2023,13 +2023,13 @@
       </c>
       <c r="W10" s="2" t="inlineStr">
         <is>
-          <t>derivacion a Alvaro Pujales, sin pregunta y sin CTA nuestro</t>
+          <t>derivación a Álvaro Pujales, sin pregunta y sin CTA nuestro</t>
         </is>
       </c>
       <c r="X10" s="2" t="inlineStr">
         <is>
-          <t>Apertura con frase de verbo, sin acuse y sin agradecimiento, para no repetir la familia de O1. Angulo verificado de su web que corrige la premisa sin contradecirle de frente. Frase de que hacemos con las palabras de base.md, empezando frase y no colgada de dos puntos. Respuesta a la objecion con el criterio de icp.md: no hace falta que monten nada, basta con pasar el pedido. Cierra derivando, porque modo.md dice que MORENO no genera cuerpo de correo comercial para este cliente y que al derivar no se calla lo que hacemos. No se ofrece llamada: activos.md tenia esa salida y modo.md la derogo el 18 de agosto. Sin margenes, sin cifras, sin prometer nada en nombre de Alvaro Pujales.
-— apertura: frase con verbo (Solo te dejo una cosa antes de cerrar) | 1ª frase: 9 palabras | qué hacemos: frase propia, verbo al inicio | cierre: derivacion sin pregunta | frases: 5</t>
+          <t>Apertura con frase de verbo, sin acuse y sin agradecimiento, para no repetir la familia de O1. Angulo verificado de su web que corrige la premisa sin contradecirle de frente. Frase de que hacemos con las palabras de base.md, empezando frase y no colgada de dos puntos. Respuesta a la objeción con el criterio de icp.md: no hace falta que monten nada, basta con pasar el pedido. Cierra derivando, porque modo.md dice que MORENO no genera cuerpo de correo comercial para este cliente y que al derivar no se calla lo que hacemos. No se ofrece llamada: activos.md tenia esa salida y modo.md la derogo el 18 de agosto. Sin márgenes, sin cifras, sin prometer nada en nombre de Álvaro Pujales.
+· apertura: frase con verbo (Solo te dejo una cosa antes de cerrar) | 1ª frase: 9 palabras | qué hacemos: frase propia, verbo al inicio | cierre: derivación sin pregunta | frases: 5</t>
         </is>
       </c>
       <c r="Y10" s="2" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>Ninguna al lead. Al derivar, estado_hilo pasa a derivada y Alvaro Pujales entra en terceros_en_hilo, y followup.md prohibe perseguir en los dos casos. El pendiente solo puede ser un recordatorio interno a Alvaro Pujales por su canal, a 2 dias laborables.</t>
+          <t>Ninguna al lead. Al derivar, estado_hilo pasa a derivada y Álvaro Pujales entra en terceros_en_hilo, y followup.md prohíbe perseguir en los dos casos. El pendiente solo puede ser un recordatorio interno a Álvaro Pujales por su canal, a 2 dias laborables.</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>Media, asi que circuito de aprobacion en Slack antes de salir, y ademas handoff_canal=ambos: plantilla del lead a Alvaro Pujales por su canal y copia en el hilo. En esta pasada en seco no sale nada.</t>
+          <t>Media, así que circuito de aprobacion en Slack antes de salir, y además handoff_canal=ambos: plantilla del lead a Álvaro Pujales por su canal y copia en el hilo. En esta pasada en seco no sale nada.</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
@@ -2174,7 +2174,7 @@
       <c r="X11" s="3" t="inlineStr">
         <is>
           <t>Sin redacción: la fase 3 de esta pasada solo redacta el grupo A. En un barrido real le tocaría cierre cordial sin push, según la matriz de metodologia.md.
-— apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
+· apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
         </is>
       </c>
       <c r="Y11" s="3" t="inlineStr">
@@ -2293,7 +2293,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>ANGULO: sin senal publica
+          <t>ANGULO: sin señal publica
 FUENTE: titus.cat, web del local, que confirma que Carpa Titus es sala de fiesta de Badalona y no restaurante de mesa
 FECHA DE LA SENAL: 
 ENCAJE: fuera
@@ -2322,7 +2322,7 @@
       <c r="X12" s="2" t="inlineStr">
         <is>
           <t>Sin redacción: la fase 3 de esta pasada solo redacta el grupo A. En real, cierre cordial de una línea y sin pedir referido, porque la empresa tampoco encaja.
-— apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
+· apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
         </is>
       </c>
       <c r="Y12" s="2" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
-          <t>ANGULO: sin senal publica
+          <t>ANGULO: sin señal publica
 FUENTE: narirestauracion.com, que se presenta como grupo de hostelería con franquicia y gestión para inversores. No hay publicación que confirme la venta de la división, solo la palabra del lead.
 FECHA DE LA SENAL: 
 ENCAJE: fuera
@@ -2468,7 +2468,7 @@
       <c r="X13" s="3" t="inlineStr">
         <is>
           <t>Sin redacción: la fase 3 de esta pasada solo redacta el grupo A. En real, cierre cordial dejando la puerta abierta por si vuelven a operar sala.
-— apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
+· apertura:  | 1ª frase: 0 palabras | qué hacemos:  | cierre:  | frases: 0</t>
         </is>
       </c>
       <c r="Y13" s="3" t="inlineStr">
@@ -2623,8 +2623,8 @@
       <c r="X14" s="4" t="inlineStr">
         <is>
           <t>circunstancial antepuesto con el volumen del lead, qué hacemos en frase propia, nombre del handoff, binaria
-— apertura: circunstancial antepuesto, sin vocativo | 1ª frase: 14 palabras | qué hacemos: frase propia con sujeto explícito | cierre: binaria | frases: 4
-— REESCRITO EN CONTROL DE LOTE: sí: la apertura original era acuse corto con vocativo (Entendido, René), la misma forma que S1 y O1</t>
+· apertura: circunstancial antepuesto, sin vocativo | 1ª frase: 14 palabras | qué hacemos: frase propia con sujeto explícito | cierre: binaria | frases: 4
+· REESCRITO EN CONTROL DE LOTE: sí: la apertura original era acuse corto con vocativo (Entendido, René), la misma forma que S1 y O1</t>
         </is>
       </c>
       <c r="Y14" s="4" t="inlineStr">
@@ -2776,7 +2776,7 @@
       <c r="X15" s="4" t="inlineStr">
         <is>
           <t>Frase con verbo que reconoce que se le ha repreguntado, el porqué del contacto anclado a una señal suya con fecha, qué hacemos entrando como subordinada causal pegada al handoff, y cierre de dos opciones. Ni acuse de una palabra ni pregunta abierta nueva.
-— apertura: frase con verbo | 1ª frase: 14 palabras | qué hacemos: subordinada | cierre: binaria de dos opciones | frases: 4</t>
+· apertura: frase con verbo | 1ª frase: 14 palabras | qué hacemos: subordinada | cierre: binaria de dos opciones | frases: 4</t>
         </is>
       </c>
       <c r="Y15" s="4" t="inlineStr">
@@ -2930,7 +2930,7 @@
       <c r="X16" s="4" t="inlineStr">
         <is>
           <t>Entrada por el dato del lead, sus cinco azoteas, el porqué anclado a algo que él mismo ha contado en prensa, qué hacemos en frase propia y handoff a Olivier con pregunta de encaje. Sin repetir el aluvión de llamadas que ya se le dijo en el M1.
-— apertura: entrada por el dato del lead | 1ª frase: 5 palabras | qué hacemos: frase propia con sujeto explícito | cierre: pregunta de encaje | frases: 5</t>
+· apertura: entrada por el dato del lead | 1ª frase: 5 palabras | qué hacemos: frase propia con sujeto explícito | cierre: pregunta de encaje | frases: 5</t>
         </is>
       </c>
       <c r="Y16" s="4" t="inlineStr">
@@ -3175,12 +3175,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Las cuentas de envio no cuadran con Supabase y ademas no cuadran entre si. Supabase declara isabel.rodriguez@offitravelteam.es y david.garcia@offitravelgroup.es. En O3 el hilo sale de isabel.rodriguez@offitravelteam.com y en O4 de isabel@offitravelteam.info. Son tres dominios distintos para el mismo cliente (.es, .com, .info) y dos alias distintos para la misma persona. Se reporta y no se corrige, segun lo indicado.</t>
+          <t>Las cuentas de envio no cuadran con Supabase y además no cuadran entre si. Supabase declara isabel.rodriguez@offitravelteam.es y david.garcia@offitravelgroup.es. En O3 el hilo sale de isabel.rodriguez@offitravelteam.com y en O4 de isabel@offitravelteam.info. Son tres dominios distintos para el mismo cliente (.es, .com, .info) y dos alias distintos para la misma persona. Se reporta y no se corrige, según lo indicado.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>datos.md prohibe deducir un identificador. Con tres candidatos, la variable de firma y el enrutado de la respuesta pueden resolverse contra la cuenta equivocada, y un hilo de Isabel acabaria firmado como otra persona o saliendo por un dominio que no es el del hilo.</t>
+          <t>datos.md prohíbe deducir un identificador. Con tres candidatos, la variable de firma y el enrutado de la respuesta pueden resolverse contra la cuenta equivocada, y un hilo de Isabel acabaria firmado como otra persona o saliendo por un dominio que no es el del hilo.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
@@ -3199,12 +3199,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>moreno_activo_desde esta en 2026-08-18 00:00 UTC y ninguno de los cuatro hilos tiene el ultimo mensaje del lead posterior a esa marca: O1 y O2 son del 17 de agosto, O3 del 2 de julio y O4 del 8 de julio. El paso 2 del motor es tajante, un hilo asi no es accionable, punto. A la vez ventana_dias=1 manda barrer desde el 17 de agosto, o sea que incluye O1 y O2.</t>
+          <t>moreno_activo_desde esta en 2026-08-18 00:00 UTC y ninguno de los cuatro hilos tiene el ultimo mensaje del lead posterior a esa marca: O1 y O2 son del 17 de agosto, O3 del 2 de julio y O4 del 8 de julio. El paso 2 del motor es tajante, un hilo así no es accionable, punto. A la vez ventana_dias=1 manda barrer desde el 17 de agosto, o sea que incluye O1 y O2.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Leido literal, la cola de este barrido es cero y se pierden dos respuestas de ayer de una campana viva (O1 y O2), que es justo lo contrario de lo que el freno pretendia (evitar escribir a hilos historicos de 2022). O3 y O4 si caen con claridad. Hace falta decidir si la fecha de corte se compara contra el inicio del dia o contra el instante, y dejarlo escrito.</t>
+          <t>Leído literal, la cola de este barrido es cero y se pierden dos respuestas de ayer de una campaña viva (O1 y O2), que es justo lo contrario de lo que el freno pretendia (evitar escribir a hilos históricos de 2022). O3 y O4 sí caen con claridad. Hace falta decidir si la fecha de corte se compara contra el inicio del dia o contra el instante, y dejarlo escrito.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
@@ -3223,12 +3223,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>El motor no cubre que un lead escriba en un idioma que el cliente no declara. voz.md seccion 0 dice que el idioma lo fija el cliente (variantes_idioma=['es_es']) y que no se infiere del lead. La seccion 1 dice que la senal del prospecto manda siempre, pero esa escalera esta escrita para elegir entre variantes del espanol, no para cambiar de idioma, y el ingles solo aparece en 6 bis como caso de MedUX. Ademas hay hecho consumado: nuestro toque del 30 de junio ya salio integro en ingles.</t>
+          <t>El motor no cubre que un lead escriba en un idioma que el cliente no declara. voz.md sección 0 dice que el idioma lo fija el cliente (variantes_idioma=['es_es']) y que no se infiere del lead. La sección 1 dice que la señal del prospecto manda siempre, pero esa escalera esta escrita para elegir entre variantes del español, no para cambiar de idioma, y el ingles solo aparece en 6 bis como caso de MedUX. Además hay hecho consumado: nuestro toque del 30 de junio ya salió integro en ingles.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Sin regla, cada barrido puede decidir distinto con el mismo hilo. Aqui no ha hecho dano porque el hilo es grupo C y no se responde, pero el siguiente lead anglofono que si sea accionable se resolvera a ojo.</t>
+          <t>Sin regla, cada barrido puede decidir distinto con el mismo hilo. Aquí no ha hecho daño porque el hilo es grupo C y no se responde, pero el siguiente lead anglofono que si sea accionable se resolvera a ojo.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
@@ -3247,12 +3247,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>modo.md de Offitravel dice que MORENO no genera cuerpo de correo para este cliente porque Alvaro Pujales escribe sus propios emails, y a la vez objetivo.md de la misma ficha declara dos senders de Instantly con su variante y su firma, y da calendario y enlace para el canal email. Leido literal, todo el inbox de email de Offitravel es derivacion obligatoria.</t>
+          <t>modo.md de Offitravel dice que MORENO no genera cuerpo de correo para este cliente porque Álvaro Pujales escribe sus propios emails, y a la vez objetivo.md de la misma ficha declara dos senders de Instantly con su variante y su firma, y da calendario y enlace para el canal email. Leído literal, todo el inbox de email de Offitravel es derivación obligatoria.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Es la regla que he aplicado en O4, que sale como derivacion en vez de como respuesta comercial. Si la intencion era prohibir solo el correo comercial de venta y no la respuesta de inbox, hoy el texto no lo dice y bloquea el canal entero, incluidos los cierres cordiales y los acuses.</t>
+          <t>Es la regla que he aplicado en O4, que sale como derivación en vez de como respuesta comercial. Si la intencion era prohibir solo el correo comercial de venta y no la respuesta de inbox, hoy el texto no lo dice y bloquea el canal entero, incluidos los cierres cordiales y los acuses.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>El primer toque del hilo, del 29 de mayo, salio vacio: Hola Joaquin, salto de linea, Un saludo, Offitravel. Es exactamente el fallo de {{icebreaker}} sin renderizar que metodologia.md seccion 2 ter documenta para EM0125 y EM0126, y este hilo es de EM0125. Encima de ese correo roto se enviaron tres toques mas.</t>
+          <t>El primer toque del hilo, del 29 de mayo, salió vacio: Hola Joaquin, salto de linea, Un saludo, Offitravel. Es exactamente el fallo de {{icebreaker}} sin renderizar que metodologia.md sección 2 ter documenta para EM0125 y EM0126, y este hilo es de EM0125. Encima de ese correo roto se enviaron tres toques mas.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>El problema es de campana, no del hilo: mientras EM0125 siga enviando ese copy sin el campo cargado, se repite con un lead nuevo cada semana. Corresponde aviso al canal del cliente, que en pasada en seco no se manda.</t>
+          <t>El problema es de campaña, no del hilo: mientras EM0125 siga enviando ese copy sin el campo cargado, se repite con un lead nuevo cada semana. Corresponde aviso al canal del cliente, que en pasada en seco no se manda.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>El toque del 1 de julio prometio lo vemos en 10 minutos. La ficha de Offitravel autoriza 15 minutos, fijado por Nico el 12 de agosto, y calendario.md dice que la duracion solo se menciona si la ficha lo autoriza y con la cifra que ella declara.</t>
+          <t>El toque del 1 de julio prometió lo vemos en 10 minutos. La ficha de Offitravel autoriza 15 minutos, fijado por Nico el 12 de agosto, y calendario.md dice que la duracion solo se menciona si la ficha lo autoriza y con la cifra que ella declara.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -3319,12 +3319,12 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>El toque del 26 de junio, identico en los dos hilos, incluye la frase Otras revenden nuestros circuitos completos bajo su propia marca. base.md la marca como error heredado de la base de conocimiento vieja y de EM0126, y declara que Offitravel no cede circuitos para que otro los revenda. Aqui ha salido por EM0125 a leads reales.</t>
+          <t>El toque del 26 de junio, identico en los dos hilos, incluye la frase Otras revenden nuestros circuitos completos bajo su propia marca. base.md la marca como error heredado de la base de conocimiento vieja y de EM0126, y declara que Offitravel no cede circuitos para que otro los revenda. Aquí ha salido por EM0125 a leads reales.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Si cualquiera de los dos leads vuelve preguntando por revender circuitos, hay que desmentir un correo propio. Ademas el mismo toque abre con la formula de reventa en dos hilos distintos, o sea que el error esta en la secuencia y no en el barrido.</t>
+          <t>Si cualquiera de los dos leads vuelve preguntando por revender circuitos, hay que desmentir un correo propio. Además el mismo toque abre con la formula de reventa en dos hilos distintos, o sea que el error esta en la secuencia y no en el barrido.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr"/>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Choque de criterio en el tag. Por el arbol de decision de tags.md, paso 17, solo vendemos habitaciones, nunca incluimos transporte es rechazo con razon estructural de modelo, o sea No Fit. Por el sub caso de Has Provider, escrito con el nombre de Offitravel dentro, esa misma objecion es una apertura y no un descarte. He aplicado Has Provider porque la ficha manda y porque el modelo no es realmente incompatible.</t>
+          <t>Choque de criterio en el tag. Por el arbol de decision de tags.md, paso 17, solo vendemos habitaciones, nunca incluimos transporte es rechazo con razon estructural de modelo, o sea No Fit. Por el sub caso de Has Provider, escrito con el nombre de Offitravel dentro, esa misma objeción es una apertura y no un descarte. He aplicado Has Provider porque la ficha manda y porque el modelo no es realmente incompatible.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>La config trae estilo_conversacion=null, o sea sin estilo declarado, mientras que objetivo.md de la ficha si define los cuatro rasgos de personalidad (quien habla, que no hace nunca, cuanto escribe, como cierra) y ademas el registro de tuteo y vosotros y el tono de disculparse por interrumpir. He redactado con la ficha.</t>
+          <t>La config trae estilo_conversacion=null, o sea sin estilo declarado, mientras que objetivo.md de la ficha si define los cuatro rasgos de personalidad (quien habla, que no hace nunca, cuanto escribe, como cierra) y además el registro de tuteo y vosotros y el tono de disculparse por interrumpir. He redactado con la ficha.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -3391,12 +3391,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Huecos de ficha aun abiertos y declarados en la propia skill: margenes para agencias, volumen minimo o condiciones de entrada, material de autoridad sin URL, y la fila en core.moreno_client_config, el canal de Slack y el barrido en modo prueba revisado por una persona sin confirmar.</t>
+          <t>Huecos de ficha aun abiertos y declarados en la propia skill: márgenes para agencias, volumen minimo o condiciones de entrada, material de autoridad sin URL, y la fila en core.moreno_client_config, el canal de Slack y el barrido en modo prueba revisado por una persona sin confirmar.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Cualquier lead que pregunte por condiciones economicas cae en derivacion obligatoria, no por criterio sino por falta de dato. Y sin material de autoridad con enlace, la rama de dejar material no tiene con que trabajar.</t>
+          <t>Cualquier lead que pregunte por condiciones economicas cae en derivación obligatoria, no por criterio sino por falta de dato. Y sin material de autoridad con enlace, la rama de dejar material no tiene con que trabajar.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr"/>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Tension entre la ficha y el motor sobre la longitud en LinkedIn. La personalidad de Offitravel dice de 1 a 3 frases, y el motor pide acuse corto, porque, que hacemos en frase propia que empiece frase (no colgada de dos puntos) y binaria de cierre, mas el tope de 25 palabras por frase. Con tres frases hay que comprimir el porque y el que hacemos en una sola.</t>
+          <t>Tensión entre la ficha y el motor sobre la longitud en LinkedIn. La personalidad de Offitravel dice de 1 a 3 frases, y el motor pide acuse corto, porque, que hacemos en frase propia que empiece frase (no colgada de dos puntos) y binaria de cierre, más el tope de 25 palabras por frase. Con tres frases hay que comprimir el porque y el que hacemos en una sola.</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Se trabajan porque esta pasada en seco lo pide de forma explícita y no escribe nada. Antes del primer barrido real hay que decidir si la fecha de corte se mueve o si estos hilos se dan por cerrados, o el barrido saldrá vacío y parecerá que no hay trabajo.</t>
+          <t>Se trabajan porque esta pasada en seco lo pide de forma explícita y no escribe nada. Antes del primer barrido real hay que decidir si la fecha de corte se mueve o sí estos hilos se dan por cerrados, o el barrido saldrá vacío y parecerá que no hay trabajo.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr"/>

</xml_diff>